<commit_message>
(documentation) reason for picking dry/wet electrodes for EMG/ECG respectively
</commit_message>
<xml_diff>
--- a/BOM/Vital-Link-BOM1-V4.xlsx
+++ b/BOM/Vital-Link-BOM1-V4.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Parry\Documents\GITHUB_desktop\Vital-link-hardware\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BC9DD7D-9458-4271-AE2A-85B69E59FCEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9D7CB97-FB7B-42C5-9178-3062F4D070A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="17385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="39">
   <si>
     <t>BOM #:</t>
   </si>
@@ -110,15 +110,6 @@
     <t>Nordic Microcontroller. Used as node</t>
   </si>
   <si>
-    <t>https://www.digikey.ca/en/products/detail/analog-devices-inc-maxim-integrated/MAXREFDES117/6165562</t>
-  </si>
-  <si>
-    <t>MAXREFDES117#</t>
-  </si>
-  <si>
-    <t>MAX1921, MAX14595, MAX30102 - Medical, Pulse Oximeter (PO or SpO2) Sensor Evaluation Board</t>
-  </si>
-  <si>
     <t>https://www.digikey.ca/en/products/detail/mikroelektronika/MIKROE-2554/7035340</t>
   </si>
   <si>
@@ -143,22 +134,22 @@
     <t>HERE'S A LIST OF ALL THE COMPONENTS on digikey</t>
   </si>
   <si>
-    <t>https://www.digikey.ca/en/products/detail/sparkfun-electronics/12650/5824153</t>
-  </si>
-  <si>
-    <t>EVAL BOARD FOR AD8232</t>
-  </si>
-  <si>
     <t>https://www.digikey.ca/en/products/detail/sparkfun-electronics/12970/6833933</t>
   </si>
   <si>
     <t>SENSOR CABLE - ELECTRODE PADS (3</t>
   </si>
   <si>
-    <t>https://www.digikey.ca/en/products/detail/sparkfun-electronics/12969/6163652</t>
-  </si>
-  <si>
-    <t>SENSOR BIOMEDICAL PADS 1=10PCS</t>
+    <t>https://www.mouser.ca/ProductDetail/DFRobot/SEN0344?qs=eP2BKZSCXI5r1K2DgtfmoA%3D%3D&amp;mgh=1&amp;srsltid=AfmBOoq-449VUTNzt2mNSoHdAZOK9qB9drzdsWTo2SL4RQDGhPqgwv0tdJw</t>
+  </si>
+  <si>
+    <t>Multiple Function Sensor Development Tools Fermion: MAX30102 PPG Heart Rate and Oximeter Sensor (Breakout, I2C/UART)</t>
+  </si>
+  <si>
+    <t>PPG</t>
+  </si>
+  <si>
+    <t>Temperature</t>
   </si>
 </sst>
 </file>
@@ -168,7 +159,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -236,6 +227,26 @@
     <font>
       <b/>
       <sz val="14"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color theme="10"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF333333"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -361,10 +372,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -372,29 +384,19 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -402,21 +404,6 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -428,12 +415,6 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -447,8 +428,41 @@
     <xf numFmtId="164" fontId="11" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -682,10 +696,10 @@
       <c r="B1" s="1">
         <v>1</v>
       </c>
-      <c r="C1" s="19" t="s">
-        <v>35</v>
-      </c>
-      <c r="D1" s="20"/>
+      <c r="C1" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="D1" s="14"/>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
@@ -699,10 +713,10 @@
       <c r="B2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="19" t="s">
-        <v>34</v>
-      </c>
-      <c r="D2" s="20"/>
+      <c r="C2" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="D2" s="14"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
@@ -710,7 +724,7 @@
       <c r="I2" s="2"/>
     </row>
     <row r="3" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="35" t="s">
+      <c r="A3" s="20" t="s">
         <v>3</v>
       </c>
       <c r="B3" s="1" t="s">
@@ -725,7 +739,7 @@
       <c r="I3" s="2"/>
     </row>
     <row r="4" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="36"/>
+      <c r="A4" s="21"/>
       <c r="B4" s="4" t="s">
         <v>5</v>
       </c>
@@ -737,7 +751,7 @@
       <c r="I4" s="2"/>
     </row>
     <row r="5" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="36"/>
+      <c r="A5" s="21"/>
       <c r="B5" s="4" t="s">
         <v>6</v>
       </c>
@@ -749,7 +763,7 @@
       <c r="I5" s="2"/>
     </row>
     <row r="6" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="37"/>
+      <c r="A6" s="22"/>
       <c r="B6" s="1" t="s">
         <v>7</v>
       </c>
@@ -803,309 +817,279 @@
       <c r="I9" s="2"/>
     </row>
     <row r="10" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="5" t="s">
+      <c r="A10" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C10" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="D10" s="29" t="s">
         <v>15</v>
       </c>
-      <c r="E10" s="5" t="s">
+      <c r="E10" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="F10" s="5" t="s">
+      <c r="F10" s="29" t="s">
         <v>17</v>
       </c>
-      <c r="G10" s="5" t="s">
+      <c r="G10" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="H10" s="5" t="s">
+      <c r="H10" s="29" t="s">
         <v>19</v>
       </c>
-      <c r="I10" s="5" t="s">
+      <c r="I10" s="29" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="7">
+      <c r="A11" s="31">
         <v>1</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="B11" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="C11" s="9" t="s">
+      <c r="C11" s="33" t="s">
         <v>22</v>
       </c>
-      <c r="D11" s="10" t="s">
+      <c r="D11" s="34" t="s">
         <v>23</v>
       </c>
-      <c r="E11" s="11">
+      <c r="E11" s="35">
         <v>3</v>
       </c>
-      <c r="F11" s="12">
+      <c r="F11" s="36">
         <v>0</v>
       </c>
-      <c r="G11" s="13">
+      <c r="G11" s="37">
         <v>15.83</v>
       </c>
-      <c r="H11" s="12">
-        <f t="shared" ref="H11" si="0">G11*E11</f>
+      <c r="H11" s="36">
+        <f t="shared" ref="H11:H15" si="0">G11*E11</f>
         <v>47.49</v>
       </c>
-      <c r="I11" s="14" t="s">
+      <c r="I11" s="34" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="7">
+      <c r="A12" s="31">
         <v>3</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="B12" s="32" t="s">
+        <v>35</v>
+      </c>
+      <c r="C12" s="38" t="s">
+        <v>36</v>
+      </c>
+      <c r="D12" s="39" t="s">
+        <v>36</v>
+      </c>
+      <c r="E12" s="35">
+        <v>1</v>
+      </c>
+      <c r="F12" s="36">
+        <v>0</v>
+      </c>
+      <c r="G12" s="36">
+        <v>24.65</v>
+      </c>
+      <c r="H12" s="36">
+        <f t="shared" si="0"/>
+        <v>24.65</v>
+      </c>
+      <c r="I12" s="40" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="31">
+        <v>4</v>
+      </c>
+      <c r="B13" s="32" t="s">
         <v>25</v>
       </c>
-      <c r="C12" s="9" t="s">
+      <c r="C13" s="33" t="s">
         <v>26</v>
       </c>
-      <c r="D12" s="14" t="s">
+      <c r="D13" s="34" t="s">
         <v>27</v>
       </c>
-      <c r="E12" s="11">
+      <c r="E13" s="35">
         <v>1</v>
       </c>
-      <c r="F12" s="12">
+      <c r="F13" s="36">
         <v>0</v>
       </c>
-      <c r="G12" s="12">
-        <v>28.08</v>
-      </c>
-      <c r="H12" s="12">
-        <f>G12*E12</f>
-        <v>28.08</v>
-      </c>
-      <c r="I12" s="14"/>
-    </row>
-    <row r="13" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="7">
-        <v>4</v>
-      </c>
-      <c r="B13" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="C13" s="23" t="s">
-        <v>29</v>
-      </c>
-      <c r="D13" s="24" t="s">
-        <v>30</v>
-      </c>
-      <c r="E13" s="25">
+      <c r="G13" s="36">
+        <v>19.2</v>
+      </c>
+      <c r="H13" s="36">
+        <f t="shared" si="0"/>
+        <v>19.2</v>
+      </c>
+      <c r="I13" s="40" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="31">
+        <v>5</v>
+      </c>
+      <c r="B14" s="42" t="s">
+        <v>33</v>
+      </c>
+      <c r="C14" s="33">
+        <v>12970</v>
+      </c>
+      <c r="D14" s="34" t="s">
+        <v>34</v>
+      </c>
+      <c r="E14" s="35">
         <v>1</v>
       </c>
-      <c r="F13" s="26">
+      <c r="F14" s="36">
         <v>0</v>
       </c>
-      <c r="G13" s="26">
-        <v>19.2</v>
-      </c>
-      <c r="H13" s="26">
-        <f>G13*E13</f>
-        <v>19.2</v>
-      </c>
-      <c r="I13" s="14"/>
-    </row>
-    <row r="14" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="21">
-        <v>5</v>
-      </c>
-      <c r="B14" s="32" t="s">
-        <v>36</v>
-      </c>
-      <c r="C14" s="34">
-        <v>12650</v>
-      </c>
-      <c r="D14" s="32" t="s">
-        <v>37</v>
-      </c>
-      <c r="E14" s="33">
-        <v>1</v>
-      </c>
-      <c r="F14" s="26">
-        <v>0</v>
-      </c>
-      <c r="G14" s="32">
-        <v>38.78</v>
-      </c>
-      <c r="H14" s="26">
-        <f t="shared" ref="H14:H16" si="1">G14*E14</f>
-        <v>38.78</v>
-      </c>
-      <c r="I14" s="22"/>
+      <c r="G14" s="36">
+        <v>14.31</v>
+      </c>
+      <c r="H14" s="36">
+        <f t="shared" si="0"/>
+        <v>14.31</v>
+      </c>
+      <c r="I14" s="34"/>
     </row>
     <row r="15" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="7">
-        <v>6</v>
-      </c>
-      <c r="B15" s="27" t="s">
-        <v>38</v>
-      </c>
-      <c r="C15" s="28">
-        <v>12970</v>
-      </c>
-      <c r="D15" s="29" t="s">
-        <v>39</v>
-      </c>
-      <c r="E15" s="30">
-        <v>1</v>
-      </c>
-      <c r="F15" s="26">
-        <v>0</v>
-      </c>
-      <c r="G15" s="31">
-        <v>14.31</v>
-      </c>
-      <c r="H15" s="26">
-        <f t="shared" si="1"/>
-        <v>14.31</v>
-      </c>
-      <c r="I15" s="14"/>
-    </row>
-    <row r="16" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="7">
-        <v>7</v>
-      </c>
-      <c r="B16" s="15" t="s">
-        <v>40</v>
-      </c>
-      <c r="C16" s="9">
-        <v>12969</v>
-      </c>
-      <c r="D16" s="14" t="s">
-        <v>41</v>
-      </c>
-      <c r="E16" s="11">
-        <v>1</v>
-      </c>
-      <c r="F16" s="26">
-        <v>0</v>
-      </c>
-      <c r="G16" s="12">
-        <v>15.81</v>
-      </c>
-      <c r="H16" s="26">
-        <f t="shared" si="1"/>
-        <v>15.81</v>
-      </c>
-      <c r="I16" s="14"/>
+      <c r="A15" s="31"/>
+      <c r="B15" s="41"/>
+      <c r="C15" s="33"/>
+      <c r="D15" s="34"/>
+      <c r="E15" s="35"/>
+      <c r="F15" s="36"/>
+      <c r="G15" s="36"/>
+      <c r="H15" s="36"/>
+      <c r="I15" s="34"/>
+    </row>
+    <row r="16" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="19"/>
+      <c r="B16" s="19"/>
+      <c r="C16" s="19"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="19"/>
+      <c r="G16" s="19"/>
+      <c r="H16" s="19"/>
+      <c r="I16" s="34"/>
     </row>
     <row r="17" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="7"/>
-      <c r="B17" s="16"/>
-      <c r="C17" s="9"/>
-      <c r="D17" s="14"/>
-      <c r="E17" s="11"/>
-      <c r="F17" s="12"/>
-      <c r="G17" s="12"/>
-      <c r="H17" s="12"/>
-      <c r="I17" s="14"/>
+      <c r="A17" s="27"/>
+      <c r="B17" s="28"/>
+      <c r="C17" s="15"/>
+      <c r="D17" s="16"/>
+      <c r="E17" s="17"/>
+      <c r="F17" s="18"/>
+      <c r="G17" s="18"/>
+      <c r="H17" s="18"/>
+      <c r="I17" s="16"/>
     </row>
     <row r="18" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="7"/>
-      <c r="B18" s="16"/>
-      <c r="C18" s="9"/>
-      <c r="D18" s="14"/>
-      <c r="E18" s="11"/>
-      <c r="F18" s="12"/>
-      <c r="G18" s="12"/>
-      <c r="H18" s="12"/>
-      <c r="I18" s="14"/>
+      <c r="A18" s="5"/>
+      <c r="B18" s="10"/>
+      <c r="C18" s="6"/>
+      <c r="D18" s="9"/>
+      <c r="E18" s="7"/>
+      <c r="F18" s="8"/>
+      <c r="G18" s="8"/>
+      <c r="H18" s="8"/>
+      <c r="I18" s="9"/>
     </row>
     <row r="19" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="7"/>
-      <c r="B19" s="16"/>
-      <c r="C19" s="9"/>
-      <c r="D19" s="14"/>
-      <c r="E19" s="11"/>
-      <c r="F19" s="12"/>
-      <c r="G19" s="12"/>
-      <c r="H19" s="12"/>
-      <c r="I19" s="14"/>
+      <c r="A19" s="5"/>
+      <c r="B19" s="10"/>
+      <c r="C19" s="6"/>
+      <c r="D19" s="9"/>
+      <c r="E19" s="7"/>
+      <c r="F19" s="8"/>
+      <c r="G19" s="8"/>
+      <c r="H19" s="8"/>
+      <c r="I19" s="9"/>
     </row>
     <row r="20" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="7"/>
-      <c r="B20" s="16"/>
-      <c r="C20" s="9"/>
-      <c r="D20" s="14"/>
-      <c r="E20" s="11"/>
-      <c r="F20" s="12"/>
-      <c r="G20" s="12"/>
-      <c r="H20" s="12"/>
-      <c r="I20" s="14"/>
+      <c r="A20" s="5"/>
+      <c r="B20" s="10"/>
+      <c r="C20" s="6"/>
+      <c r="D20" s="9"/>
+      <c r="E20" s="7"/>
+      <c r="F20" s="8"/>
+      <c r="G20" s="8"/>
+      <c r="H20" s="8"/>
+      <c r="I20" s="9"/>
     </row>
     <row r="21" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="7"/>
-      <c r="B21" s="16"/>
-      <c r="C21" s="9"/>
-      <c r="D21" s="14"/>
-      <c r="E21" s="11"/>
-      <c r="F21" s="12"/>
-      <c r="G21" s="12"/>
-      <c r="H21" s="12"/>
-      <c r="I21" s="14"/>
+      <c r="A21" s="5"/>
+      <c r="B21" s="10"/>
+      <c r="C21" s="6"/>
+      <c r="D21" s="9"/>
+      <c r="E21" s="7"/>
+      <c r="F21" s="8"/>
+      <c r="G21" s="8"/>
+      <c r="H21" s="8"/>
+      <c r="I21" s="9"/>
     </row>
     <row r="22" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="4"/>
-      <c r="C22" s="17"/>
+      <c r="C22" s="11"/>
       <c r="D22" s="4"/>
-      <c r="E22" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="F22" s="38">
+      <c r="E22" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="F22" s="23">
         <f>SUM(H11:H21)</f>
-        <v>163.67000000000002</v>
-      </c>
-      <c r="G22" s="39"/>
-      <c r="H22" s="40"/>
+        <v>105.65</v>
+      </c>
+      <c r="G22" s="24"/>
+      <c r="H22" s="25"/>
       <c r="I22" s="4"/>
     </row>
     <row r="23" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="4"/>
-      <c r="C23" s="17"/>
+      <c r="C23" s="11"/>
       <c r="D23" s="4"/>
-      <c r="E23" s="18" t="s">
-        <v>32</v>
-      </c>
-      <c r="F23" s="38">
+      <c r="E23" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="F23" s="23">
         <f>F22*0.12</f>
-        <v>19.6404</v>
-      </c>
-      <c r="G23" s="39"/>
-      <c r="H23" s="40"/>
+        <v>12.678000000000001</v>
+      </c>
+      <c r="G23" s="24"/>
+      <c r="H23" s="25"/>
       <c r="I23" s="4"/>
     </row>
     <row r="24" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="4"/>
       <c r="B24" s="4"/>
-      <c r="C24" s="17"/>
+      <c r="C24" s="11"/>
       <c r="D24" s="4"/>
-      <c r="E24" s="18" t="s">
-        <v>33</v>
-      </c>
-      <c r="F24" s="41">
+      <c r="E24" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="F24" s="26">
         <f>SUM(F22:H23)</f>
-        <v>183.31040000000002</v>
-      </c>
-      <c r="G24" s="39"/>
-      <c r="H24" s="40"/>
+        <v>118.328</v>
+      </c>
+      <c r="G24" s="24"/>
+      <c r="H24" s="25"/>
       <c r="I24" s="4"/>
     </row>
     <row r="25" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="4"/>
       <c r="B25" s="4"/>
-      <c r="C25" s="17"/>
+      <c r="C25" s="11"/>
       <c r="D25" s="4"/>
       <c r="E25" s="4"/>
       <c r="F25" s="4"/>
@@ -1122,9 +1106,10 @@
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="B11" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="B12" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="B13" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="B13" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="B14" r:id="rId3" xr:uid="{393FD92E-BB69-41B0-8530-923917FBF429}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId4"/>
 </worksheet>
 </file>
</xml_diff>